<commit_message>
Add official Gibraltar Registry fee table, DIY totals and visa finding to tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xq11JveUnH4mTddeupkfHp
</commit_message>
<xml_diff>
--- a/Gibraltar_wedding_2026_v1.xlsx
+++ b/Gibraltar_wedding_2026_v1.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Offer &amp; Terms" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Documents" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Open Questions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Next Steps" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Official Fees" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Documents" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Open Questions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Next Steps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;€&quot;#,##0"/>
+    <numFmt numFmtId="166" formatCode="&quot;£&quot;#,##0"/>
+  </numFmts>
   <fonts count="7">
     <font>
       <name val="Calibri"/>
@@ -104,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -120,6 +125,13 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,6 +519,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -695,6 +708,8 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
@@ -774,7 +789,7 @@
       <c r="B23" s="10" t="n"/>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Not stated in the offer. Confirm whether the 3-course meal is included in the fee.</t>
+          <t>See 'Official Fees' sheet for Registry and Botanic Gardens fees. Harbour restaurant meal cost still not stated.</t>
         </is>
       </c>
     </row>
@@ -804,6 +819,417 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Gibraltar Registry fees (official) and do-it-yourself totals</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Source: Civil Status &amp; Registration Office, Ceremony Guidance Notes fee table (screenshot supplied by Lisa, 24 Sep 2026). Blue = official figure; black = formula; yellow = to confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Fee item</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Registrar's Certificate (residents only)</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Not applicable to non-residents</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Notice (residents only)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Not applicable to non-residents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Special Licence for Marriage</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>124</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Required for non-residents</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Ceremony at the Registry Office</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>186.5</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Weekdays only</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Ceremony at an Outside Location</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>309.5</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>After working hours on weekdays, and Saturdays</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Mayor's Parlour venue fee</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>372</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Separate fee charged by Cultural Services, in addition to the ceremony fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Marriage Certificate (each)</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>37</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Issued 10 to 15 working days after the ceremony</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Confirmation Letter</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Provided immediately after the ceremony on the day</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Postage of certificates outside Gibraltar</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Apostille (each)</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>37</v>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Placed on the reverse of the certificate; needed for recognition in China, check for UK</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Change of Date fee</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>53</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Only if the date is moved</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Botanic Gardens 'The Dell' hire, weekday</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="n">
+        <v>275</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Alameda Gardens price list; season 1 Apr to 30 Oct; confirm 2026 price with events@gibraltargardens.gi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Botanic Gardens 'The Dell' hire, Saturday</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>As above</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Do-it-yourself totals (what Marry Abroad Simply's fee replaces)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>What is included</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Registry Office, bare minimum</t>
+        </is>
+      </c>
+      <c r="B21" s="13">
+        <f>B7+B8+B11</f>
+        <v/>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Special Licence, ceremony at Registry, one certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Registry Office, with letter, postage and apostille</t>
+        </is>
+      </c>
+      <c r="B22" s="13">
+        <f>B7+B8+B11+B12+B13+B14</f>
+        <v/>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>As above plus confirmation letter on the day, postage to UK, one apostille</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Botanic Gardens, weekday evening</t>
+        </is>
+      </c>
+      <c r="B23" s="13">
+        <f>B7+B9+B16+B11+B12+B13+B14</f>
+        <v/>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Special Licence, outside-location ceremony, Dell hire, certificate, letter, postage, apostille</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Botanic Gardens, Saturday</t>
+        </is>
+      </c>
+      <c r="B24" s="13">
+        <f>B7+B9+B17+B11+B12+B13+B14</f>
+        <v/>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>As above with Saturday Dell hire</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Harbour restaurant (venue and meal not known)</t>
+        </is>
+      </c>
+      <c r="B25" s="13">
+        <f>B7+B9+B11+B12+B13+B14</f>
+        <v/>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Government fees only; add the restaurant's own charge</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Comparison with Marry Abroad Simply</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Agency fee EUR</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="n">
+        <v>1495</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Agency fee GBP (agency's own quoted equivalent)</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Marry Abroad Simply advertises Gibraltar at EUR 1,495 / GBP 1,250. Confirm the exact GBP charge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Agency premium over Botanic Gardens weekday DIY</t>
+        </is>
+      </c>
+      <c r="B30" s="17">
+        <f>B29-B23</f>
+        <v/>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>What you pay the agency for document checking, booking and being your contact. Venue is included in their fee; the meal at the harbour restaurant may not be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Agency premium over Registry Office DIY (with extras)</t>
+        </is>
+      </c>
+      <c r="B31" s="17">
+        <f>B29-B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Not included in any total: flights London to Gibraltar, at least one hotel night (required), certified translations, Chinese single-status notarisation, Schengen visa fee (about EUR 90) and any meal.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1223,7 +1649,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1311,11 +1737,19 @@
           <t>This was dropped from the email sent on 18 Sep and never asked.</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Since 15 Jul 2026 Gibraltar follows Schengen short-stay visa rules. UK residence/visa exemption ended. Chinese citizens need a Schengen visa, applied for via Spain (BLS London) when Gibraltar is the main destination. BLS requires the UK residence permit to be valid 90 days beyond the return date. Lisa's UK visa ends Dec 2026, so an application from London for an October trip is likely to be refused. Also, Registry guidance requires UK residents to show a share code with at least 6 months validity.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Blocking</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1822,11 @@
           <t>Deposit is non-refundable in this case because the Denmark risk was flagged. Confirm whether a deposit already paid for Denmark transfers.</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Official Registry fees now known, see 'Official Fees' sheet. Agency deposit/payment timing still to confirm.</t>
+        </is>
+      </c>
       <c r="F8" s="4" t="inlineStr"/>
       <c r="G8" s="4" t="inlineStr">
         <is>
@@ -1478,7 +1916,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Record Gibraltar option as not feasible for Oct 2026 after visa and residence checks
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xq11JveUnH4mTddeupkfHp
</commit_message>
<xml_diff>
--- a/Gibraltar_wedding_2026_v1.xlsx
+++ b/Gibraltar_wedding_2026_v1.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +132,9 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -519,7 +522,13 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
+    <row r="3" ht="75" customHeight="1">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>STATUS 24 Sep 2026: Gibraltar is not feasible for Sep/Oct 2026. Lisa's UK Graduate (PSW) visa expires 20 Dec 2026, so (a) her share code fails the Registry's 6-month residence rule and (b) BLS Spain in London will not take a Schengen visa application unless the UK permit is valid 90 days beyond the return date. Andreas (British, German, Romanian) needs no visa. Couple relocating to San Francisco around end Oct 2026, so a later Gibraltar date does not help.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -708,8 +717,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
@@ -1739,7 +1746,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Since 15 Jul 2026 Gibraltar follows Schengen short-stay visa rules. UK residence/visa exemption ended. Chinese citizens need a Schengen visa, applied for via Spain (BLS London) when Gibraltar is the main destination. BLS requires the UK residence permit to be valid 90 days beyond the return date. Lisa's UK visa ends Dec 2026, so an application from London for an October trip is likely to be refused. Also, Registry guidance requires UK residents to show a share code with at least 6 months validity.</t>
+          <t>Since 15 Jul 2026 Gibraltar follows Schengen short-stay visa rules. UK residence/visa exemption ended. Chinese citizens need a Schengen visa, applied for via Spain (BLS London) when Gibraltar is the main destination. BLS requires the UK residence permit to be valid 90 days beyond the return date. Lisa's UK visa ends Dec 2026, so an application from London for an October trip is likely to be refused. Also, Registry guidance requires UK residents to show a share code with at least 6 months validity. Confirmed 24 Sep: Lisa holds a Graduate (PSW) visa valid to 20 Dec 2026; Andreas is a British, German and Romanian citizen and needs no visa. Lisa holds no Schengen visa as far as known. Conclusion: no realistic route to enter and marry in Gibraltar before the end-October move.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -1749,7 +1756,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Blocking</t>
+          <t>Closed - blocks option</t>
         </is>
       </c>
     </row>
@@ -1946,6 +1953,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Superseded 24 Sep 2026: Gibraltar option parked. The couple is giving notice at Camden Town Hall instead; that is tracked separately.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Close Gibraltar option: single-entry Schengen visa already used
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xq11JveUnH4mTddeupkfHp
</commit_message>
<xml_diff>
--- a/Gibraltar_wedding_2026_v1.xlsx
+++ b/Gibraltar_wedding_2026_v1.xlsx
@@ -522,10 +522,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="75" customHeight="1">
+    <row r="3" ht="95" customHeight="1">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>STATUS 24 Sep 2026: Gibraltar is not feasible for Sep/Oct 2026. Lisa's UK Graduate (PSW) visa expires 20 Dec 2026, so (a) her share code fails the Registry's 6-month residence rule and (b) BLS Spain in London will not take a Schengen visa application unless the UK permit is valid 90 days beyond the return date. Andreas (British, German, Romanian) needs no visa. Couple relocating to San Francisco around end Oct 2026, so a later Gibraltar date does not help.</t>
+          <t>STATUS 30 Sep 2026: GIBRALTAR CLOSED. Lisa's only Schengen visa (Portugal, type C, single entry, 5 days, valid 18 Sep to 7 Oct 2026) was used for the Faro trip of 25 to 29 Sep 2026, so she cannot re-enter the Schengen area or Gibraltar before it expires. A new Schengen visa cannot be issued from London because her UK permit ends 20 Dec 2026. Marry Abroad Simply's 7 Oct slot was also gone by 30 Sep. Remaining options: Camden Town Hall (notice given 23 Sep, earliest ceremony 22 Oct) or Georgia (visa-free for Chinese and British citizens).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Note Camden ceremony booked and Home Office referral concluded
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xq11JveUnH4mTddeupkfHp
</commit_message>
<xml_diff>
--- a/Gibraltar_wedding_2026_v1.xlsx
+++ b/Gibraltar_wedding_2026_v1.xlsx
@@ -522,10 +522,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="95" customHeight="1">
+    <row r="3" ht="120" customHeight="1">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>STATUS 30 Sep 2026: GIBRALTAR CLOSED. Lisa's only Schengen visa (Portugal, type C, single entry, 5 days, valid 18 Sep to 7 Oct 2026) was used for the Faro trip of 25 to 29 Sep 2026, so she cannot re-enter the Schengen area or Gibraltar before it expires. A new Schengen visa cannot be issued from London because her UK permit ends 20 Dec 2026. Marry Abroad Simply's 7 Oct slot was also gone by 30 Sep. Remaining options: Camden Town Hall (notice given 23 Sep, earliest ceremony 22 Oct) or Georgia (visa-free for Chinese and British citizens).</t>
+          <t>STATUS 30 Sep 2026: GIBRALTAR CLOSED. Lisa's only Schengen visa (Portugal, type C, single entry, 5 days, valid 18 Sep to 7 Oct 2026) was used for the Faro trip of 25 to 29 Sep 2026, so she cannot re-enter the Schengen area or Gibraltar before it expires. A new Schengen visa cannot be issued from London because her UK permit ends 20 Dec 2026. Marry Abroad Simply's 7 Oct slot was also gone by 30 Sep. Remaining options: Camden Town Hall (notice given 23 Sep, earliest ceremony 22 Oct) or Georgia (visa-free for Chinese and British citizens). UPDATE 1 Oct 2026: Home Office confirmed no investigation; free to marry after the 28 days. Camden Town Hall, Primrose Room, booked for Thursday 22 Oct 2026 at 10:15 (booking ID 10034679). Gibraltar track closed.</t>
         </is>
       </c>
     </row>

</xml_diff>